<commit_message>
dicionario, coneitual, modelo logico
</commit_message>
<xml_diff>
--- a/modelo_dicionario_de_dados.xlsx
+++ b/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="100">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -109,6 +109,21 @@
   </si>
   <si>
     <t xml:space="preserve">equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHAVE PRIMÁRIA DE IDENTIFICAÇÃO DO EQUIPAMENTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHAVE PRIMÁRIA DE IDENTIFICAÇÃO DO CARGO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHAVE PRIMÁRIA DE IDENTIFICAÇÃO DA SITUACAO</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -984,7 +999,7 @@
       </c>
       <c r="H14" s="7"/>
       <c r="I14" s="15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1007,45 +1022,89 @@
       <c r="I15" s="14"/>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="8"/>
+      <c r="A16" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="8"/>
+      <c r="E16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>22</v>
+      </c>
       <c r="H16" s="7"/>
-      <c r="I16" s="10"/>
+      <c r="I16" s="15" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="12"/>
+      <c r="A17" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
+      <c r="F17" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G17" s="12"/>
       <c r="H17" s="11"/>
       <c r="I17" s="14"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="8"/>
+      <c r="A18" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="8"/>
+      <c r="E18" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>22</v>
+      </c>
       <c r="H18" s="7"/>
-      <c r="I18" s="10"/>
+      <c r="I18" s="15" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
+      <c r="A19" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
+      <c r="F19" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G19" s="12"/>
       <c r="H19" s="11"/>
       <c r="I19" s="14"/>
@@ -1535,89 +1594,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1625,7 +1684,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>10</v>
@@ -1640,10 +1699,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>16</v>
@@ -1651,16 +1710,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>20</v>
@@ -1669,160 +1728,160 @@
         <v>21</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C19" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D19" s="13" t="s">
-        <v>55</v>
-      </c>
       <c r="E19" s="13" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C20" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="9" t="s">
         <v>67</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>62</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>20</v>
@@ -1831,65 +1890,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1919,15 +1978,15 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>21</v>
@@ -1935,23 +1994,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1961,27 +2020,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>